<commit_message>
Correct heat-detector note after GENT product research
The workbook previously called the RFP's "S4 VAD addressable heat
detector" a specification error on the grounds that VAD means visual
alarm device. That was wrong: Gent builds heat sensors with an
integrated VAD strobe (S4-720-V-VAD-HPR / -HPW), so the wording
describes a real product.

The clarification still matters, for a different reason. At 57,000 to
76,000 per unit these lines are priced below the plain sounder-VAD
lines at 90,000 to 145,000, which suggests bidders priced ordinary heat
sensors rather than the VAD variant.

Also adds notes confirming every Gent part number quoted is a real
current product, and flagging that loop loading needs a proper
calculation rather than a device count.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TrsGsn5u798GV9DGHsoozh
</commit_message>
<xml_diff>
--- a/Projects/Ikeja City Mall Fire Alarm/ICM_Fire_Alarm_Bid_Comparison.xlsx
+++ b/Projects/Ikeja City Mall Fire Alarm/ICM_Fire_Alarm_Bid_Comparison.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="209">
   <si>
     <t xml:space="preserve">IKEJA CITY MALL - FIRE DETECTION &amp; ALARM SYSTEM OVERHAUL</t>
   </si>
@@ -199,7 +199,7 @@
     <t xml:space="preserve">GENT S4 "VAD" addressable heat detectors</t>
   </si>
   <si>
-    <t xml:space="preserve">RFP wording "S4 VAD heat detector" is a spec error - VAD = visual alarm device, not a heat detector. All 5 bids repeat it. Clarify before award.</t>
+    <t xml:space="preserve">Gent does make heat sensors with an integrated VAD strobe (S4-720-V-VAD-HPR / -HPW), so the RFP wording describes a real product. But at 57,000-76,000 these lines are priced like PLAIN heat sensors - below the sounder-VAD lines at 90,000-145,000. Confirm which variant is being supplied before award.</t>
   </si>
   <si>
     <t xml:space="preserve">GENT S4-34842 addressable manual call points (MCPs)</t>
@@ -603,10 +603,22 @@
     <t xml:space="preserve">Roundbox's total is roughly half the GENT bids because it substitutes TANDA equipment throughout - e.g. a smoke detector at ~20,600 delivered against 57,000-76,000 for GENT. The RFP requires equipment compatible with the existing GENT Vigilon system, so this is a rip-and-replace alternative, not a cheaper version of the tendered work. It is excluded from the compliant-bid ranking.</t>
   </si>
   <si>
-    <t xml:space="preserve">Specification defect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The RFP asks for 60 "GENT S4 VAD Addressable Heat Detectors". VAD means visual alarm device (strobe), not a heat detector. All five bids repeat the wording without query. Clarify before award - it affects 60 units of pricing.</t>
+    <t xml:space="preserve">Heat detector variant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The RFP asks for 60 "GENT S4 VAD Addressable Heat Detectors". Gent does build heat sensors with an integrated visual alarm device (S4-720-V-VAD-HPR red / -HPW white), so the wording is valid. The concern is pricing: at 57,000-76,000 per unit these lines sit below the plain sounder-VAD lines (90,000-145,000), which suggests bidders priced ordinary heat sensors rather than the VAD variant. Worth 60 units of clarification before award.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part numbers verified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every Gent part number appearing in the bids is a real, current product: Vigilon Plus 24 panel, S4-715 optical smoke, S4-710 optical/heat multi-sensor, S4-720 heat, S4-700 common base, S4-34842 manual call point (EN54-11, with cover), and S3-S-VAD-HPR-R sounder/VAD from the S-Cubed range (EN54-23, Vigilon compatible). No bidder invented a part.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loop loading</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vigilon Plus supports 200 devices per loop, so 540 devices over 4 loops plus the expansion panel is within capacity on device count. Gent also applies a load factor per device type (a manual call point counts 4) and limits sounder-VADs to about 70 per loop, so the winning contractor must produce a proper loop loading calculation, not just a device count.</t>
   </si>
   <si>
     <t xml:space="preserve">Loop capacity</t>
@@ -3948,7 +3960,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -4087,7 +4099,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="n">
         <v>11</v>
       </c>
@@ -4098,7 +4110,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="n">
         <v>12</v>
       </c>
@@ -4109,7 +4121,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="n">
         <v>13</v>
       </c>
@@ -4120,7 +4132,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="n">
         <v>14</v>
       </c>
@@ -4131,7 +4143,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="n">
         <v>15</v>
       </c>
@@ -4142,29 +4154,51 @@
         <v>199</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
+    <row r="20" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="47" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="50" t="s">
+      <c r="C20" s="6" t="s">
         <v>201</v>
       </c>
     </row>
+    <row r="21" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="47" t="s">
+        <v>202</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="51" t="s">
-        <v>202</v>
+      <c r="A23" s="18" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="52" t="s">
-        <v>203</v>
+      <c r="B24" s="50" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="53" t="s">
-        <v>204</v>
+      <c r="B25" s="51" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="52" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="53" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>